<commit_message>
Fix XSS vulnerabilities and remove withdrawn medicine (Ranitidine)
Co-authored-by: mj11rock <23415371+mj11rock@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/medicines.xlsx
+++ b/medicines.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -824,44 +824,44 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ranitidine</t>
+          <t>Ciprofloxacin</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ranitidine</t>
+          <t>Ciprofloxacin</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>H2 Blocker</t>
+          <t>Antibiotic</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Reduces stomach acid</t>
+          <t>Fluoroquinolone antibiotic</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>150mg twice daily</t>
+          <t>250mg-750mg twice daily</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Headache, constipation, diarrhea</t>
+          <t>Nausea, diarrhea, dizziness</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ciprofloxacin</t>
+          <t>Azithromycin</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ciprofloxacin</t>
+          <t>Azithromycin</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -871,162 +871,162 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Fluoroquinolone antibiotic</t>
+          <t>Macrolide antibiotic</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>250mg-750mg twice daily</t>
+          <t>500mg on day 1, then 250mg daily</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Nausea, diarrhea, dizziness</t>
+          <t>Diarrhea, nausea, stomach pain</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Azithromycin</t>
+          <t>Prednisone</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Azithromycin</t>
+          <t>Prednisone</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Antibiotic</t>
+          <t>Corticosteroid</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Macrolide antibiotic</t>
+          <t>Reduces inflammation</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>500mg on day 1, then 250mg daily</t>
+          <t>5mg-60mg daily</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Diarrhea, nausea, stomach pain</t>
+          <t>Increased appetite, mood changes, insomnia</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Prednisone</t>
+          <t>Insulin</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prednisone</t>
+          <t>Insulin</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Corticosteroid</t>
+          <t>Hormone</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Reduces inflammation</t>
+          <t>Blood sugar control for diabetes</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>5mg-60mg daily</t>
+          <t>Varies by type and patient needs</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Increased appetite, mood changes, insomnia</t>
+          <t>Low blood sugar, weight gain</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Insulin</t>
+          <t>Warfarin</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Insulin</t>
+          <t>Warfarin</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hormone</t>
+          <t>Anticoagulant</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Blood sugar control for diabetes</t>
+          <t>Blood thinner</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Varies by type and patient needs</t>
+          <t>Varies based on INR monitoring</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Low blood sugar, weight gain</t>
+          <t>Bleeding, bruising</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Warfarin</t>
+          <t>Losartan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Warfarin</t>
+          <t>Losartan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Anticoagulant</t>
+          <t>ARB</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Blood thinner</t>
+          <t>Blood pressure medication</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Varies based on INR monitoring</t>
+          <t>25mg-100mg once daily</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bleeding, bruising</t>
+          <t>Dizziness, fatigue, back pain</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Losartan</t>
+          <t>Amlodipine</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Losartan</t>
+          <t>Amlodipine</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ARB</t>
+          <t>Calcium Channel Blocker</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1036,74 +1036,42 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>25mg-100mg once daily</t>
+          <t>5mg-10mg once daily</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Dizziness, fatigue, back pain</t>
+          <t>Swelling, dizziness, flushing</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Amlodipine</t>
+          <t>Gabapentin</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Amlodipine</t>
+          <t>Gabapentin</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Calcium Channel Blocker</t>
+          <t>Anticonvulsant</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Blood pressure medication</t>
+          <t>Treats nerve pain and seizures</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5mg-10mg once daily</t>
+          <t>300mg-3600mg daily in divided doses</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
-        <is>
-          <t>Swelling, dizziness, flushing</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Gabapentin</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Gabapentin</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Anticonvulsant</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Treats nerve pain and seizures</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>300mg-3600mg daily in divided doses</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
         <is>
           <t>Dizziness, drowsiness, fatigue</t>
         </is>

</xml_diff>